<commit_message>
feat: implement modular test automation framework for retail operations with Selenium and Excel integration
</commit_message>
<xml_diff>
--- a/Sparqla/Sqarqla_Retail_data2.xlsx
+++ b/Sparqla/Sqarqla_Retail_data2.xlsx
@@ -1,78 +1,79 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7635" tabRatio="600" firstSheet="47" activeTab="49" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Login" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metal" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CategoryName" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SubDesign" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Designmapping" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subdesignmapping" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MC&amp;VA" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lot_Lwt" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lot_othermetal" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag_LWt" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag_othermetal" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EST" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag_EST" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NonTag_Est" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HomeBill_Est" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HomeBill_Lwt" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OldMetal_Est" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oldmetal_Lwt" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendor" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contract_Price" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stone_price" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kyc" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer_LWT" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Billing" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Credit_Card" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cheque" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NetBanking" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SALES" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SALES &amp; PURCHASE" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SALES PURCHASE &amp; RETURN" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PURCHASE" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ORDER ADVANCE" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SALES RETURN" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CREDIT COLLECTION" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ORDER DELIVERY" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHIT PRE CLOSE" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Receipt" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PurchasePO" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PurchasePO_Items" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GRNEntry" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GRNEntry_Items" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SupplierBillEntry" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SupplierBillEntry_Items" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SupplierPOPayment" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MetalPocket" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ApprovalRateFixing" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ApprovalRateFixingItems" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SearchBill" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BillingIssue" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BillingReceipt" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AdvanceTransfer" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OldMetalProcess" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RepairOrderStatus" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InventoryCategory" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PackagingItemSize" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OtherInventory" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductMapping" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductPurchaseEntry" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PackagingItemIssue" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OtherInventoryTagging" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="Master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Login" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Metal" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CategoryName" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Product" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Design" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="SubDesign" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Designmapping" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Subdesignmapping" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="MC&amp;VA" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Lot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Lot_Lwt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Lot_othermetal" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Tag" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Tag_LWt" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Tag_othermetal" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="EST" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Tag_EST" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="NonTag_Est" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="HomeBill_Est" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="HomeBill_Lwt" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="OldMetal_Est" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Oldmetal_Lwt" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Vendor" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Contract_Price" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Stone_price" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Kyc" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Customer" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Customer_LWT" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Billing" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Credit_Card" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="Cheque" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="NetBanking" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="SALES" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="SALES &amp; PURCHASE" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="SALES PURCHASE &amp; RETURN" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="PURCHASE" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="ORDER ADVANCE" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="SALES RETURN" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="CREDIT COLLECTION" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="ORDER DELIVERY" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="CHIT PRE CLOSE" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="Issue" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="Receipt" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="PurchasePO" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="PurchasePO_Items" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="GRNEntry" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="GRNEntry_Items" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="SupplierBillEntry" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="SupplierBillEntry_Items" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="SupplierPOPayment" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="MetalPocket" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="ApprovalRateFixing" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="ApprovalRateFixingItems" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="SearchBill" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="BillingIssue" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="BillingReceipt" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="AdvanceTransfer" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="OldMetalProcess" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="RepairOrderStatus" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="InventoryCategory" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="PackagingItemSize" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="OtherInventory" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="ProductMapping" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="ProductPurchaseEntry" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="PackagingItemIssue" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="OtherInventoryTagging" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="ApprovalToInvoice" sheetId="68" state="visible" r:id="rId68"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Product'!$A$1:$AF$136</definedName>
@@ -86,7 +87,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="54">
+  <fonts count="55">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -413,8 +414,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -461,6 +466,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF4472C4"/>
         <bgColor rgb="FF4472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
       </patternFill>
     </fill>
   </fills>
@@ -597,7 +608,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -727,6 +738,7 @@
     <xf numFmtId="0" fontId="53" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="54" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -37426,7 +37438,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
     </row>
@@ -57454,8 +57466,6 @@
           <t>Enable</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Product Details Added successfully</t>
@@ -57473,11 +57483,105 @@
           <t>Enable</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Product Details Added successfully</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="87" t="inlineStr">
+        <is>
+          <t>TestCaseId</t>
+        </is>
+      </c>
+      <c r="B1" s="87" t="inlineStr">
+        <is>
+          <t>TestStatus</t>
+        </is>
+      </c>
+      <c r="C1" s="87" t="inlineStr">
+        <is>
+          <t>ActualStatus</t>
+        </is>
+      </c>
+      <c r="D1" s="87" t="inlineStr">
+        <is>
+          <t>OpeningBal</t>
+        </is>
+      </c>
+      <c r="E1" s="87" t="inlineStr">
+        <is>
+          <t>RateCutType</t>
+        </is>
+      </c>
+      <c r="F1" s="87" t="inlineStr">
+        <is>
+          <t>ConvertTo</t>
+        </is>
+      </c>
+      <c r="G1" s="87" t="inlineStr">
+        <is>
+          <t>ConvType</t>
+        </is>
+      </c>
+      <c r="H1" s="87" t="inlineStr">
+        <is>
+          <t>SupplierName</t>
+        </is>
+      </c>
+      <c r="I1" s="87" t="inlineStr">
+        <is>
+          <t>RefNo</t>
+        </is>
+      </c>
+      <c r="J1" s="87" t="inlineStr">
+        <is>
+          <t>Metal</t>
+        </is>
+      </c>
+      <c r="K1" s="87" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="L1" s="87" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="M1" s="87" t="inlineStr">
+        <is>
+          <t>PureWeight</t>
+        </is>
+      </c>
+      <c r="N1" s="87" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="O1" s="87" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="P1" s="87" t="inlineStr">
+        <is>
+          <t>Remark</t>
         </is>
       </c>
     </row>

</xml_diff>